<commit_message>
Validated the foorprints for the PCB
</commit_message>
<xml_diff>
--- a/Excel/Charger.xlsx
+++ b/Excel/Charger.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uoa-my.sharepoint.com/personal/msun711_uoa_auckland_ac_nz/Documents/Desktop/311/Excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="139" documentId="11_F25DC773A252ABDACC104819191F4C6C5ADE58E9" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{57D0A254-6B14-4A88-9AD0-DD0A0328D721}"/>
+  <xr:revisionPtr revIDLastSave="221" documentId="11_F25DC773A252ABDACC104819191F4C6C5ADE58E9" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5A095CAF-0563-4029-B793-948A6CB5D512}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
   <si>
     <t xml:space="preserve">BJT </t>
   </si>
@@ -39,9 +39,6 @@
     <t>Rg</t>
   </si>
   <si>
-    <t>Rb</t>
-  </si>
-  <si>
     <t>Ra</t>
   </si>
   <si>
@@ -63,15 +60,6 @@
     <t>Rsense</t>
   </si>
   <si>
-    <t>Calcuation:</t>
-  </si>
-  <si>
-    <t>Low side sensing was chosen to throw out the high common Mode Voltage. Hnece no IC is required for the current sensor. </t>
-  </si>
-  <si>
-    <t>A gain of 100 is selected: so that when R = 0.1, and from our smulation, a maximum of 0.2A is reached. There fore(0.2*0.1)*100 = 2V. </t>
-  </si>
-  <si>
     <t>Mosfet</t>
   </si>
   <si>
@@ -84,17 +72,38 @@
     <t>Rc</t>
   </si>
   <si>
-    <t>Rd</t>
-  </si>
-  <si>
     <t>Co</t>
+  </si>
+  <si>
+    <t>Diode</t>
+  </si>
+  <si>
+    <t>CMOZ1l8</t>
+  </si>
+  <si>
+    <t>Battery</t>
+  </si>
+  <si>
+    <t>Opamp</t>
+  </si>
+  <si>
+    <t>TLV9162</t>
+  </si>
+  <si>
+    <t>D1</t>
+  </si>
+  <si>
+    <t>We have to buy it</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+  </numFmts>
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -107,6 +116,20 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -126,17 +149,22 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Currency" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -419,174 +447,219 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:O21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="E1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="G2">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>0</v>
       </c>
       <c r="C3" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="G3">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>1</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" s="1"/>
+      <c r="E4" s="1"/>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C5" s="1"/>
+      <c r="E5" s="1">
         <v>1000</v>
       </c>
-      <c r="G4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B5" t="s">
+      <c r="G5">
         <v>3</v>
       </c>
-      <c r="C5" s="1">
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" s="1"/>
+      <c r="E6" s="1">
         <v>1000</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" s="1">
-        <v>1000</v>
-      </c>
-      <c r="E6" s="1"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="1">
+      <c r="C7" s="1"/>
+      <c r="E7" s="1">
         <v>1000</v>
       </c>
-      <c r="E7" s="1"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C8" s="1">
-        <v>5600</v>
-      </c>
-      <c r="E8" s="1"/>
+        <v>10</v>
+      </c>
+      <c r="C8" s="1"/>
+      <c r="E8" s="1">
+        <v>1</v>
+      </c>
       <c r="G8">
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>19</v>
-      </c>
-      <c r="C9" s="1">
-        <v>3300</v>
-      </c>
-      <c r="G9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+      <c r="C9" s="1"/>
+      <c r="E9" s="1">
+        <v>120</v>
+      </c>
+      <c r="G9" s="4">
+        <v>1</v>
+      </c>
+      <c r="K9" s="1"/>
+      <c r="M9" s="1"/>
+      <c r="O9">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>11</v>
-      </c>
-      <c r="C10" s="1">
-        <v>1</v>
-      </c>
-      <c r="G10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+      <c r="C10" s="1"/>
+      <c r="E10" s="1">
+        <v>47000</v>
+      </c>
+      <c r="G10" s="4">
+        <v>1</v>
+      </c>
+      <c r="K10" s="1"/>
+      <c r="M10" s="1"/>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>16</v>
+      </c>
       <c r="C11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="G11" s="1"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G11" s="3"/>
+      <c r="I11" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="J11" s="5"/>
+      <c r="K11" s="1"/>
+      <c r="M11" s="1"/>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>21</v>
+      </c>
       <c r="C12" s="1"/>
-      <c r="G12" s="1"/>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E12" t="s">
+        <v>17</v>
+      </c>
+      <c r="G12">
+        <v>1</v>
+      </c>
+      <c r="K12" s="1"/>
+      <c r="M12" s="1"/>
+      <c r="O12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>5</v>
+      </c>
       <c r="C13" s="1"/>
-    </row>
-    <row r="14" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C14" s="1"/>
-    </row>
-    <row r="15" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G13" s="1"/>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>9</v>
+      </c>
+      <c r="E14" s="1">
+        <v>3.3E-10</v>
+      </c>
+      <c r="G14" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
+        <v>8</v>
+      </c>
       <c r="C15" s="1"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>6</v>
-      </c>
+      <c r="E15" s="1">
+        <v>4.6999999999999999E-6</v>
+      </c>
+      <c r="G15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>10</v>
-      </c>
-      <c r="C16" s="1"/>
-      <c r="G16" s="1">
-        <v>4.7000000000000003E-10</v>
+        <v>15</v>
+      </c>
+      <c r="E16" s="1">
+        <v>1E-4</v>
+      </c>
+      <c r="G16">
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>9</v>
-      </c>
-      <c r="G17" s="1">
-        <v>9.9999999999999995E-8</v>
+        <v>18</v>
+      </c>
+      <c r="E17" s="1">
+        <v>30</v>
+      </c>
+      <c r="G17">
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B18" t="s">
+      <c r="A18" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B19" t="s">
         <v>20</v>
       </c>
-      <c r="C18" s="1"/>
-      <c r="G18">
-        <v>1</v>
-      </c>
+      <c r="G19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="2"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="2" t="s">
-        <v>14</v>
-      </c>
+      <c r="A21" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Added components list in charger spreadsheet
</commit_message>
<xml_diff>
--- a/Excel/Charger.xlsx
+++ b/Excel/Charger.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pacopoon/Downloads/311/Excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB1CE93D-3718-7D47-B99A-04A9E23604A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F407F742-0412-CF4C-B544-67C4B9923741}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4800" yWindow="660" windowWidth="25440" windowHeight="17240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4800" yWindow="660" windowWidth="25440" windowHeight="17240" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Specifications" sheetId="2" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="1" r:id="rId2"/>
+    <sheet name="Components" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,75 +26,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="70">
-  <si>
-    <t xml:space="preserve">BJT </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Resistor </t>
-  </si>
-  <si>
-    <t>Rf1</t>
-  </si>
-  <si>
-    <t>Rg</t>
-  </si>
-  <si>
-    <t>Ra</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="65">
   <si>
     <t>Capacitor</t>
-  </si>
-  <si>
-    <t>Quality</t>
   </si>
   <si>
     <t>Value</t>
   </si>
   <si>
-    <t>Ca</t>
-  </si>
-  <si>
-    <t>Zf</t>
-  </si>
-  <si>
-    <t>Rsense</t>
-  </si>
-  <si>
-    <t>Mosfet</t>
-  </si>
-  <si>
     <t>IRF9Z24N</t>
-  </si>
-  <si>
-    <t>BD180</t>
-  </si>
-  <si>
-    <t>Rc</t>
-  </si>
-  <si>
-    <t>Co</t>
-  </si>
-  <si>
-    <t>Diode</t>
-  </si>
-  <si>
-    <t>CMOZ1l8</t>
-  </si>
-  <si>
-    <t>Battery</t>
-  </si>
-  <si>
-    <t>Opamp</t>
-  </si>
-  <si>
-    <t>TLV9162</t>
-  </si>
-  <si>
-    <t>D1</t>
-  </si>
-  <si>
-    <t>We have to buy it</t>
   </si>
   <si>
     <t>Charger Design - Part I</t>
@@ -236,6 +176,51 @@
   </si>
   <si>
     <t>This is lower than the T_junction max in the datasheet (175) but should still use heatsink</t>
+  </si>
+  <si>
+    <t>OPAMP</t>
+  </si>
+  <si>
+    <t>Component</t>
+  </si>
+  <si>
+    <t>Part Number</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>TLV9162IDR</t>
+  </si>
+  <si>
+    <t>Zener diode</t>
+  </si>
+  <si>
+    <t>CMOZ1L8</t>
+  </si>
+  <si>
+    <t>PNP BJT</t>
+  </si>
+  <si>
+    <t>BD140</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PMOS </t>
+  </si>
+  <si>
+    <t>Resistor</t>
+  </si>
+  <si>
+    <t>470nF</t>
+  </si>
+  <si>
+    <t>1uF</t>
+  </si>
+  <si>
+    <t>3.3nF</t>
+  </si>
+  <si>
+    <t>47k</t>
   </si>
 </sst>
 </file>
@@ -400,7 +385,7 @@
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -419,6 +404,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Check Cell" xfId="2" builtinId="23"/>
@@ -714,7 +700,7 @@
   <sheetData>
     <row r="1" spans="1:26" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -771,7 +757,7 @@
     </row>
     <row r="3" spans="1:26" ht="19" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="B3" s="6"/>
       <c r="C3" s="6"/>
@@ -828,13 +814,13 @@
     </row>
     <row r="5" spans="1:26" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A5" s="11" t="s">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="D5" s="6"/>
       <c r="E5" s="6"/>
@@ -862,13 +848,13 @@
     </row>
     <row r="6" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A6" s="12" t="s">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="B6" s="13">
         <v>5</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="D6" s="6"/>
       <c r="E6" s="6"/>
@@ -896,13 +882,13 @@
     </row>
     <row r="7" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A7" s="12" t="s">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="B7" s="13">
         <v>3.5</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="D7" s="6"/>
       <c r="E7" s="6"/>
@@ -930,13 +916,13 @@
     </row>
     <row r="8" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A8" s="12" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="B8" s="13">
         <v>0</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="D8" s="6"/>
       <c r="E8" s="6"/>
@@ -964,13 +950,13 @@
     </row>
     <row r="9" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A9" s="12" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="B9" s="13">
         <v>0.17499999999999999</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="D9" s="6"/>
       <c r="E9" s="6"/>
@@ -998,13 +984,13 @@
     </row>
     <row r="10" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A10" s="12" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="B10" s="13">
         <v>0.5</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>33</v>
+        <v>13</v>
       </c>
       <c r="D10" s="6"/>
       <c r="E10" s="6"/>
@@ -1032,13 +1018,13 @@
     </row>
     <row r="11" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A11" s="12" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="B11" s="13">
         <v>1.75</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="D11" s="6"/>
       <c r="E11" s="6"/>
@@ -1066,13 +1052,13 @@
     </row>
     <row r="12" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A12" s="12" t="s">
-        <v>36</v>
+        <v>16</v>
       </c>
       <c r="B12" s="13">
         <v>0.875</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="D12" s="6"/>
       <c r="E12" s="6"/>
@@ -1100,13 +1086,13 @@
     </row>
     <row r="13" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A13" s="12" t="s">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="B13" s="13">
         <v>183.75</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="D13" s="6"/>
       <c r="E13" s="6"/>
@@ -1134,13 +1120,13 @@
     </row>
     <row r="14" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A14" s="12" t="s">
-        <v>39</v>
+        <v>19</v>
       </c>
       <c r="B14" s="13">
         <v>210</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="D14" s="6"/>
       <c r="E14" s="6"/>
@@ -1196,7 +1182,7 @@
     </row>
     <row r="16" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A16" s="10" t="s">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="B16" s="6"/>
       <c r="C16" s="6"/>
@@ -1254,7 +1240,7 @@
     </row>
     <row r="18" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A18" s="8" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
@@ -1284,7 +1270,7 @@
     </row>
     <row r="19" spans="1:26" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>43</v>
+        <v>23</v>
       </c>
       <c r="B19" s="6"/>
       <c r="C19" s="6"/>
@@ -1314,13 +1300,13 @@
     </row>
     <row r="20" spans="1:26" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A20" s="11" t="s">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="D20" s="6"/>
       <c r="E20" s="6"/>
@@ -1348,18 +1334,18 @@
     </row>
     <row r="21" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A21" s="12" t="s">
-        <v>44</v>
+        <v>24</v>
       </c>
       <c r="B21" s="13">
         <v>0.25</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="D21" s="6"/>
       <c r="E21" s="6"/>
       <c r="F21" s="8" t="s">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="G21" s="6"/>
       <c r="H21" s="6"/>
@@ -1384,18 +1370,18 @@
     </row>
     <row r="22" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A22" s="12" t="s">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="B22" s="13">
         <v>52.5</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="D22" s="6"/>
       <c r="E22" s="6"/>
       <c r="F22" s="8" t="s">
-        <v>47</v>
+        <v>27</v>
       </c>
       <c r="G22" s="6"/>
       <c r="H22" s="6"/>
@@ -1448,10 +1434,10 @@
     </row>
     <row r="24" spans="1:26" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A24" s="8" t="s">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>49</v>
+        <v>29</v>
       </c>
       <c r="C24" s="6"/>
       <c r="D24" s="6"/>
@@ -1477,18 +1463,18 @@
     </row>
     <row r="25" spans="1:26" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A25" s="11" t="s">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="D25" s="6"/>
       <c r="E25" s="6"/>
       <c r="F25" s="8" t="s">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="G25" s="6"/>
       <c r="H25" s="6"/>
@@ -1511,18 +1497,18 @@
     </row>
     <row r="26" spans="1:26" ht="16" x14ac:dyDescent="0.2">
       <c r="A26" s="12" t="s">
-        <v>51</v>
+        <v>31</v>
       </c>
       <c r="B26" s="13">
         <v>4.5</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="D26" s="6"/>
       <c r="E26" s="6"/>
       <c r="F26" s="9" t="s">
-        <v>52</v>
+        <v>32</v>
       </c>
       <c r="G26" s="6"/>
       <c r="H26" s="6"/>
@@ -1545,18 +1531,18 @@
     </row>
     <row r="27" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A27" s="12" t="s">
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="B27" s="13">
         <v>1</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="D27" s="6"/>
       <c r="E27" s="6"/>
       <c r="F27" s="10" t="s">
-        <v>54</v>
+        <v>34</v>
       </c>
       <c r="G27" s="6"/>
       <c r="H27" s="6"/>
@@ -1607,18 +1593,18 @@
     </row>
     <row r="29" spans="1:26" ht="16" x14ac:dyDescent="0.2">
       <c r="A29" s="12" t="s">
-        <v>55</v>
+        <v>35</v>
       </c>
       <c r="B29" s="13">
         <v>2.25</v>
       </c>
       <c r="C29" s="13" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="D29" s="6"/>
       <c r="E29" s="6"/>
       <c r="F29" s="9" t="s">
-        <v>56</v>
+        <v>36</v>
       </c>
       <c r="G29" s="6"/>
       <c r="H29" s="6"/>
@@ -1641,18 +1627,18 @@
     </row>
     <row r="30" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A30" s="12" t="s">
-        <v>57</v>
+        <v>37</v>
       </c>
       <c r="B30" s="13">
         <v>0.5</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="D30" s="6"/>
       <c r="E30" s="6"/>
       <c r="F30" s="10" t="s">
-        <v>58</v>
+        <v>38</v>
       </c>
       <c r="G30" s="6"/>
       <c r="H30" s="6"/>
@@ -1675,13 +1661,13 @@
     </row>
     <row r="31" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A31" s="12" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="B31" s="13">
         <v>1.375</v>
       </c>
       <c r="C31" s="13" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="D31" s="6"/>
       <c r="E31" s="6"/>
@@ -1709,13 +1695,13 @@
     </row>
     <row r="32" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A32" s="12" t="s">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="B32" s="13">
         <v>288.75</v>
       </c>
       <c r="C32" s="13" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="D32" s="6"/>
       <c r="E32" s="6"/>
@@ -1771,7 +1757,7 @@
     </row>
     <row r="34" spans="1:26" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A34" s="8" t="s">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="B34" s="6"/>
       <c r="C34" s="6"/>
@@ -1801,13 +1787,13 @@
     </row>
     <row r="35" spans="1:26" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A35" s="11" t="s">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="B35" s="11" t="s">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C35" s="11" t="s">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="D35" s="6"/>
       <c r="E35" s="6"/>
@@ -1835,13 +1821,13 @@
     </row>
     <row r="36" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A36" s="12" t="s">
-        <v>61</v>
+        <v>41</v>
       </c>
       <c r="B36" s="13">
         <v>1.75</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="D36" s="6"/>
       <c r="E36" s="6"/>
@@ -1869,13 +1855,13 @@
     </row>
     <row r="37" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A37" s="12" t="s">
-        <v>62</v>
+        <v>42</v>
       </c>
       <c r="B37" s="13">
         <v>0</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="D37" s="6"/>
       <c r="E37" s="6"/>
@@ -1903,13 +1889,13 @@
     </row>
     <row r="38" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A38" s="12" t="s">
-        <v>63</v>
+        <v>43</v>
       </c>
       <c r="B38" s="13">
         <v>0.875</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="D38" s="6"/>
       <c r="E38" s="6"/>
@@ -1937,13 +1923,13 @@
     </row>
     <row r="39" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A39" s="12" t="s">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="B39" s="13">
         <v>183.75</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="D39" s="6"/>
       <c r="E39" s="6"/>
@@ -1999,7 +1985,7 @@
     </row>
     <row r="41" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A41" s="6" t="s">
-        <v>68</v>
+        <v>48</v>
       </c>
       <c r="B41" s="6"/>
       <c r="C41" s="6"/>
@@ -2029,13 +2015,13 @@
     </row>
     <row r="42" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A42" s="12" t="s">
-        <v>64</v>
+        <v>44</v>
       </c>
       <c r="B42" s="12">
         <v>525</v>
       </c>
       <c r="C42" s="12" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="D42" s="6"/>
       <c r="E42" s="6"/>
@@ -2062,13 +2048,13 @@
     </row>
     <row r="43" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A43" s="12" t="s">
-        <v>65</v>
+        <v>45</v>
       </c>
       <c r="B43" s="12">
         <v>525</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="D43" s="6"/>
       <c r="E43" s="6"/>
@@ -2123,13 +2109,13 @@
     </row>
     <row r="45" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A45" s="12" t="s">
-        <v>66</v>
+        <v>46</v>
       </c>
       <c r="B45" s="13">
         <v>164.5</v>
       </c>
       <c r="C45" s="13" t="s">
-        <v>67</v>
+        <v>47</v>
       </c>
       <c r="D45" s="6"/>
       <c r="E45" s="6"/>
@@ -2158,7 +2144,7 @@
     <row r="46" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A46" s="6"/>
       <c r="B46" s="6" t="s">
-        <v>69</v>
+        <v>49</v>
       </c>
       <c r="C46" s="6"/>
       <c r="D46" s="6"/>
@@ -28904,218 +28890,170 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O21"/>
+  <dimension ref="A2:M21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="E1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>11</v>
+    <row r="2" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B2" t="s">
+        <v>51</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>52</v>
       </c>
-      <c r="G2">
+      <c r="D2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>0</v>
+      <c r="E2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="3" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B3" t="s">
+        <v>50</v>
       </c>
       <c r="C3" t="s">
-        <v>13</v>
+        <v>54</v>
       </c>
-      <c r="G3">
+      <c r="E3">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+    <row r="4" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E4" s="16">
         <v>1</v>
       </c>
-      <c r="C4" s="1"/>
-      <c r="E4" s="1"/>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+    </row>
+    <row r="5" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
+        <v>57</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E5" s="16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B6" t="s">
+        <v>59</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="1"/>
-      <c r="E5" s="1">
+      <c r="E6" s="16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C7" s="1"/>
+      <c r="D7">
+        <v>1.5</v>
+      </c>
+      <c r="E7" s="16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B8" t="s">
+        <v>60</v>
+      </c>
+      <c r="C8" s="1"/>
+      <c r="D8">
         <v>1000</v>
       </c>
-      <c r="G5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="B6" t="s">
-        <v>3</v>
-      </c>
-      <c r="C6" s="1"/>
-      <c r="E6" s="1">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="B7" t="s">
+      <c r="E8" s="16">
         <v>4</v>
       </c>
-      <c r="C7" s="1"/>
-      <c r="E7" s="1">
-        <v>1000</v>
+    </row>
+    <row r="9" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B9" t="s">
+        <v>60</v>
       </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="B8" t="s">
-        <v>10</v>
+      <c r="D9" t="s">
+        <v>64</v>
       </c>
-      <c r="C8" s="1"/>
-      <c r="E8" s="1">
-        <v>1</v>
-      </c>
-      <c r="G8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="B9" t="s">
-        <v>3</v>
-      </c>
-      <c r="C9" s="1"/>
-      <c r="E9" s="1">
-        <v>120</v>
-      </c>
-      <c r="G9">
+      <c r="E9" s="16">
         <v>1</v>
       </c>
       <c r="K9" s="1"/>
       <c r="M9" s="1"/>
-      <c r="O9">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+    </row>
+    <row r="10" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B10" t="s">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="C10" s="1"/>
-      <c r="E10" s="1">
-        <v>47000</v>
+      <c r="D10" t="s">
+        <v>61</v>
       </c>
-      <c r="G10">
+      <c r="E10" s="16">
         <v>1</v>
       </c>
       <c r="K10" s="1"/>
       <c r="M10" s="1"/>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>16</v>
+    <row r="11" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B11" t="s">
+        <v>0</v>
       </c>
       <c r="C11" s="1"/>
+      <c r="D11" t="s">
+        <v>62</v>
+      </c>
+      <c r="E11" s="16">
+        <v>1</v>
+      </c>
       <c r="G11" s="3"/>
-      <c r="I11" s="4" t="s">
-        <v>22</v>
-      </c>
+      <c r="I11" s="4"/>
       <c r="J11" s="4"/>
       <c r="K11" s="1"/>
       <c r="M11" s="1"/>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B12" t="s">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="C12" s="1"/>
-      <c r="E12" t="s">
-        <v>17</v>
+      <c r="D12" t="s">
+        <v>63</v>
       </c>
-      <c r="G12">
+      <c r="E12" s="16">
         <v>1</v>
       </c>
       <c r="K12" s="1"/>
       <c r="M12" s="1"/>
-      <c r="O12">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>5</v>
-      </c>
+    </row>
+    <row r="13" spans="2:13" x14ac:dyDescent="0.2">
       <c r="C13" s="1"/>
       <c r="G13" s="1"/>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="B14" t="s">
-        <v>9</v>
-      </c>
-      <c r="E14" s="1">
-        <v>3.3E-10</v>
-      </c>
-      <c r="G14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="B15" t="s">
-        <v>8</v>
-      </c>
+    <row r="14" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="C14" s="1"/>
+    </row>
+    <row r="15" spans="2:13" x14ac:dyDescent="0.2">
       <c r="C15" s="1"/>
-      <c r="E15" s="1">
-        <v>4.6999999999999999E-6</v>
-      </c>
-      <c r="G15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="B16" t="s">
-        <v>15</v>
-      </c>
-      <c r="E16" s="1">
-        <v>1E-4</v>
-      </c>
-      <c r="G16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B17" t="s">
-        <v>18</v>
-      </c>
-      <c r="E17" s="1">
-        <v>30</v>
-      </c>
-      <c r="G17">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B19" t="s">
-        <v>20</v>
-      </c>
-      <c r="G19">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="E15" s="1"/>
+    </row>
+    <row r="16" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="E16" s="1"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E17" s="1"/>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" s="2"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" s="2"/>
     </row>
   </sheetData>

</xml_diff>